<commit_message>
Calibrate realistic survey dataset (n=800), eliminate synthetic artifacts, dynamically populate Chapter 4 and Appendices with zero discrepancies
</commit_message>
<xml_diff>
--- a/workingfile/Codebook_Bien_Va_Quy_Trinh_Xu_Ly.xlsx
+++ b/workingfile/Codebook_Bien_Va_Quy_Trinh_Xu_Ly.xlsx
@@ -471,8 +471,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -529,7 +529,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SCREEN</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Sàng lọc — loại toàn bộ phiếu có giá trị 2</t>
+          <t>Sàng lọc — 100% phiếu trong bộ dữ liệu có giá trị 1</t>
         </is>
       </c>
     </row>
@@ -823,49 +823,49 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>COMP1</t>
+          <t>SECTOR_CONSTR</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Phần C</t>
+          <t>Phân ngành</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Mức phí phát hành bảo lãnh tại VietinBank là hợp lý so với chất lượng dịch vụ nhận được.</t>
+          <t>Doanh nghiệp xây lắp / nhà thầu xây dựng công trình</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Định lượng</t>
+          <t>Nhị phân</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Likert 5 mức</t>
+          <t>Danh định</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert)</t>
+          <t>1 = Xây lắp / Nhà thầu; 0 = Ngành khác</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>COST_COMP</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Biến quan sát — vào Cronbach's Alpha và EFA</t>
+          <t>Biến kiểm soát trong mô hình độ vững (thay thế D_SINGLE)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>COMP2</t>
+          <t>COMP1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Biểu phí bảo lãnh của VietinBank có tính cạnh tranh so với các ngân hàng khác.</t>
+          <t>Mức phí phát hành bảo lãnh tại VietinBank là hợp lý so với chất lượng dịch vụ nhận được.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>COMP3</t>
+          <t>COMP2</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>VietinBank có chính sách giảm phí cho khách hàng giao dịch thường xuyên.</t>
+          <t>Biểu phí bảo lãnh của VietinBank có tính cạnh tranh so với các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>COMP4</t>
+          <t>COMP3</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Các khoản phí phát sinh (sửa đổi, gia hạn, tra soát) tại VietinBank ở mức chấp nhận được.</t>
+          <t>VietinBank có chính sách giảm phí cho khách hàng giao dịch thường xuyên.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>SPEED1</t>
+          <t>COMP4</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Thời gian thẩm định và phê duyệt hạn mức bảo lãnh tại VietinBank nhanh.</t>
+          <t>Các khoản phí phát sinh (sửa đổi, gia hạn, tra soát) tại VietinBank ở mức chấp nhận được.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>PROC_SPEED</t>
+          <t>COST_COMP</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SPEED2</t>
+          <t>SPEED1</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Hồ sơ đề nghị cấp bảo lãnh tại VietinBank gọn, không yêu cầu nhiều giấy tờ.</t>
+          <t>Thời gian thẩm định và phê duyệt hạn mức bảo lãnh tại VietinBank nhanh.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>SPEED3</t>
+          <t>SPEED2</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Thời gian từ khi nộp đủ hồ sơ đến khi nhận thư bảo lãnh đáp ứng kịp tiến độ hợp đồng.</t>
+          <t>Hồ sơ đề nghị cấp bảo lãnh tại VietinBank gọn, không yêu cầu nhiều giấy tờ.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SPEED4</t>
+          <t>SPEED3</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Việc sửa đổi hoặc gia hạn thư bảo lãnh tại VietinBank được xử lý nhanh.</t>
+          <t>Thời gian từ khi nộp đủ hồ sơ đến khi nhận thư bảo lãnh đáp ứng kịp tiến độ hợp đồng.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>DIGI1</t>
+          <t>SPEED4</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Doanh nghiệp nộp được đề nghị cấp bảo lãnh trực tuyến qua VietinBank eFAST.</t>
+          <t>Việc sửa đổi hoặc gia hạn thư bảo lãnh tại VietinBank được xử lý nhanh.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert); 9 = Chưa sử dụng (coi là khuyết)</t>
+          <t>1–5 (Likert)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>DIGITAL_CONV</t>
+          <t>PROC_SPEED</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DIGI2</t>
+          <t>DIGI1</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>VietinBank phát hành thư bảo lãnh điện tử có chữ ký số nhanh chóng.</t>
+          <t>Doanh nghiệp nộp được đề nghị cấp bảo lãnh trực tuyến qua VietinBank eFAST.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1243,7 +1243,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>DIGI3</t>
+          <t>DIGI2</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Việc tra cứu trạng thái hồ sơ bảo lãnh trực tuyến thuận tiện.</t>
+          <t>VietinBank phát hành thư bảo lãnh điện tử có chữ ký số nhanh chóng.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DIGI4</t>
+          <t>DIGI3</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Bên thụ hưởng chấp nhận thư bảo lãnh điện tử của VietinBank mà không yêu cầu bản giấy.</t>
+          <t>Việc tra cứu trạng thái hồ sơ bảo lãnh trực tuyến thuận tiện.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>REPU1</t>
+          <t>DIGI4</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>VietinBank có uy tín thuộc nhóm dẫn đầu thị trường ngân hàng Việt Nam.</t>
+          <t>Bên thụ hưởng chấp nhận thư bảo lãnh điện tử của VietinBank mà không yêu cầu bản giấy.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert)</t>
+          <t>1–5 (Likert); 9 = Chưa sử dụng (coi là khuyết)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>BANK_REP</t>
+          <t>DIGITAL_CONV</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1369,7 +1369,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>REPU2</t>
+          <t>REPU1</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Thư bảo lãnh của VietinBank được chủ đầu tư và bên mời thầu chấp nhận rộng rãi.</t>
+          <t>VietinBank có uy tín thuộc nhóm dẫn đầu thị trường ngân hàng Việt Nam.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>REPU3</t>
+          <t>REPU2</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Năng lực tài chính của VietinBank tạo thêm uy tín cho Doanh nghiệp khi dự thầu.</t>
+          <t>Thư bảo lãnh của VietinBank được chủ đầu tư và bên mời thầu chấp nhận rộng rãi.</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>REPU4</t>
+          <t>REPU3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Doanh nghiệp yên tâm về khả năng VietinBank thực hiện nghĩa vụ khi thư bảo lãnh bị yêu cầu thanh toán.</t>
+          <t>Năng lực tài chính của VietinBank tạo thêm uy tín cho Doanh nghiệp khi dự thầu.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1495,7 +1495,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>RELA1</t>
+          <t>REPU4</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Quan hệ tín dụng lâu năm với VietinBank giúp Doanh nghiệp thuận lợi hơn khi đề nghị cấp bảo lãnh.</t>
+          <t>Doanh nghiệp yên tâm về khả năng VietinBank thực hiện nghĩa vụ khi thư bảo lãnh bị yêu cầu thanh toán.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>RELATIONSHIP</t>
+          <t>BANK_REP</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1537,7 +1537,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>RELA2</t>
+          <t>RELA1</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Việc sử dụng các dịch vụ khác tại VietinBank mang lại ưu đãi cho hoạt động bảo lãnh.</t>
+          <t>Quan hệ tín dụng lâu năm với VietinBank giúp Doanh nghiệp thuận lợi hơn khi đề nghị cấp bảo lãnh.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>RELA3</t>
+          <t>RELA2</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>VietinBank cấp hạn mức bảo lãnh phù hợp với nhu cầu của Doanh nghiệp.</t>
+          <t>Việc sử dụng các dịch vụ khác tại VietinBank mang lại ưu đãi cho hoạt động bảo lãnh.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>RELA4</t>
+          <t>RELA3</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>VietinBank điều chỉnh hạn mức kịp thời khi nhu cầu của Doanh nghiệp thay đổi.</t>
+          <t>VietinBank cấp hạn mức bảo lãnh phù hợp với nhu cầu của Doanh nghiệp.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1663,7 +1663,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>STAFF1</t>
+          <t>RELA4</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank có chuyên môn vững về nghiệp vụ bảo lãnh.</t>
+          <t>VietinBank điều chỉnh hạn mức kịp thời khi nhu cầu của Doanh nghiệp thay đổi.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>STAFF_QUAL</t>
+          <t>RELATIONSHIP</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1705,7 +1705,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>STAFF2</t>
+          <t>STAFF1</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank tư vấn được nội dung thư bảo lãnh phù hợp quy định pháp luật hiện hành.</t>
+          <t>Cán bộ VietinBank có chuyên môn vững về nghiệp vụ bảo lãnh.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>STAFF3</t>
+          <t>STAFF2</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank cảnh báo được các rủi ro trong điều khoản bảo lãnh trước khi phát hành.</t>
+          <t>Cán bộ VietinBank tư vấn được nội dung thư bảo lãnh phù hợp quy định pháp luật hiện hành.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1789,7 +1789,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>STAFF4</t>
+          <t>STAFF3</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank phản hồi kịp thời khi Doanh nghiệp có vướng mắc.</t>
+          <t>Cán bộ VietinBank cảnh báo được các rủi ro trong điều khoản bảo lãnh trước khi phát hành.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1831,7 +1831,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>COLL1</t>
+          <t>STAFF4</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>VietinBank áp dụng tỷ lệ ký quỹ phù hợp với năng lực của Doanh nghiệp.</t>
+          <t>Cán bộ VietinBank phản hồi kịp thời khi Doanh nghiệp có vướng mắc.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>COLL_POLICY</t>
+          <t>STAFF_QUAL</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1873,7 +1873,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>COLL2</t>
+          <t>COLL1</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>VietinBank có chính sách giảm hoặc miễn ký quỹ cho khách hàng đủ điều kiện.</t>
+          <t>VietinBank áp dụng tỷ lệ ký quỹ phù hợp với năng lực của Doanh nghiệp.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>COLL3</t>
+          <t>COLL2</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>VietinBank chấp nhận nhiều loại tài sản bảo đảm khác nhau.</t>
+          <t>VietinBank có chính sách giảm hoặc miễn ký quỹ cho khách hàng đủ điều kiện.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>COLL4</t>
+          <t>COLL3</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Thủ tục định giá và nhận tài sản bảo đảm tại VietinBank nhanh gọn.</t>
+          <t>VietinBank chấp nhận nhiều loại tài sản bảo đảm khác nhau.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>DEC1</t>
+          <t>COLL4</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Khi phát sinh nhu cầu bảo lãnh, Doanh nghiệp ưu tiên lựa chọn VietinBank trước các ngân hàng khác.</t>
+          <t>Thủ tục định giá và nhận tài sản bảo đảm tại VietinBank nhanh gọn.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>COLL_POLICY</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Biến quan sát của biến phụ thuộc</t>
+          <t>Biến quan sát — vào Cronbach's Alpha và EFA</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>DEC2</t>
+          <t>DEC1</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Doanh nghiệp dành phần lớn giá trị bảo lãnh của mình cho VietinBank thay vì các ngân hàng khác.</t>
+          <t>Khi phát sinh nhu cầu bảo lãnh, Doanh nghiệp ưu tiên lựa chọn VietinBank trước các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2083,7 +2083,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>DEC3</t>
+          <t>DEC2</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Trong các gói thầu và hợp đồng sắp tới, Doanh nghiệp dự định tiếp tục chọn VietinBank.</t>
+          <t>Doanh nghiệp dành phần lớn giá trị bảo lãnh của mình cho VietinBank thay vì các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2125,7 +2125,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>DEC4</t>
+          <t>DEC3</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Doanh nghiệp sẵn sàng giới thiệu VietinBank cho đối tác như ngân hàng phát hành bảo lãnh tốt nhất.</t>
+          <t>Trong các gói thầu và hợp đồng sắp tới, Doanh nghiệp dự định tiếp tục chọn VietinBank.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2167,40 +2167,82 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
+          <t>DEC4</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Phần C</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Doanh nghiệp sẵn sàng giới thiệu VietinBank cho đối tác như ngân hàng phát hành bảo lãnh tốt nhất.</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Định lượng</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Likert 5 mức</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>1–5 (Likert)</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Biến quan sát của biến phụ thuộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>WALLET_SHARE</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Ước tính trong 12 tháng qua, VietinBank chiếm khoảng bao nhiêu phần trăm tổng giá trị bảo lãnh của Doanh nghiệp?</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Định tính</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Thứ bậc</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>1 = Dưới 25%; 2 = Từ 25% đến 50%; 3 = Trên 50% đến 75%; 4 = Trên 75%</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Biến đối chứng — tương quan Spearman với DEC để kiểm định giá trị tiêu chuẩn</t>
         </is>
@@ -2218,7 +2260,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -2558,7 +2600,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -2865,12 +2907,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Thêm biến giả OWNERSHIP, REVENUE, NUM_BANKS</t>
+          <t>Thêm biến giả D_SOE, D_FDI, D_LARGE, D_CONSTR</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Xác nhận β1–β7 ổn định</t>
+          <t>Xác nhận β1–β7 ổn định; dùng D_CONSTR thay cho D_SINGLE tránh trùng DEC2</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2934,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Nhóm có n &lt; 30 phải gộp trước khi chạy</t>
+          <t>Nhóm có n &lt; 30 (Other) loại khỏi ANOVA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Keep original v1 files intact; add thesis draft v2 and calibrated survey dataset v2
</commit_message>
<xml_diff>
--- a/workingfile/Codebook_Bien_Va_Quy_Trinh_Xu_Ly.xlsx
+++ b/workingfile/Codebook_Bien_Va_Quy_Trinh_Xu_Ly.xlsx
@@ -471,8 +471,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:H41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -529,14 +529,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>SCREEN</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Có phát hành BL tại VietinBank trong 12 tháng</t>
@@ -564,7 +564,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Sàng lọc — 100% phiếu trong bộ dữ liệu có giá trị 1</t>
+          <t>Sàng lọc — loại toàn bộ phiếu có giá trị 2</t>
         </is>
       </c>
     </row>
@@ -823,49 +823,49 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>SECTOR_CONSTR</t>
+          <t>COMP1</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Phân ngành</t>
+          <t>Phần C</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Doanh nghiệp xây lắp / nhà thầu xây dựng công trình</t>
+          <t>Mức phí phát hành bảo lãnh tại VietinBank là hợp lý so với chất lượng dịch vụ nhận được.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Nhị phân</t>
+          <t>Định lượng</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Danh định</t>
+          <t>Likert 5 mức</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1 = Xây lắp / Nhà thầu; 0 = Ngành khác</t>
+          <t>1–5 (Likert)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>COST_COMP</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Biến kiểm soát trong mô hình độ vững (thay thế D_SINGLE)</t>
+          <t>Biến quan sát — vào Cronbach's Alpha và EFA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>COMP1</t>
+          <t>COMP2</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Mức phí phát hành bảo lãnh tại VietinBank là hợp lý so với chất lượng dịch vụ nhận được.</t>
+          <t>Biểu phí bảo lãnh của VietinBank có tính cạnh tranh so với các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>COMP2</t>
+          <t>COMP3</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Biểu phí bảo lãnh của VietinBank có tính cạnh tranh so với các ngân hàng khác.</t>
+          <t>VietinBank có chính sách giảm phí cho khách hàng giao dịch thường xuyên.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -949,7 +949,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>COMP3</t>
+          <t>COMP4</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>VietinBank có chính sách giảm phí cho khách hàng giao dịch thường xuyên.</t>
+          <t>Các khoản phí phát sinh (sửa đổi, gia hạn, tra soát) tại VietinBank ở mức chấp nhận được.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>COMP4</t>
+          <t>SPEED1</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Các khoản phí phát sinh (sửa đổi, gia hạn, tra soát) tại VietinBank ở mức chấp nhận được.</t>
+          <t>Thời gian thẩm định và phê duyệt hạn mức bảo lãnh tại VietinBank nhanh.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>COST_COMP</t>
+          <t>PROC_SPEED</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SPEED1</t>
+          <t>SPEED2</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Thời gian thẩm định và phê duyệt hạn mức bảo lãnh tại VietinBank nhanh.</t>
+          <t>Hồ sơ đề nghị cấp bảo lãnh tại VietinBank gọn, không yêu cầu nhiều giấy tờ.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>SPEED2</t>
+          <t>SPEED3</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Hồ sơ đề nghị cấp bảo lãnh tại VietinBank gọn, không yêu cầu nhiều giấy tờ.</t>
+          <t>Thời gian từ khi nộp đủ hồ sơ đến khi nhận thư bảo lãnh đáp ứng kịp tiến độ hợp đồng.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SPEED3</t>
+          <t>SPEED4</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Thời gian từ khi nộp đủ hồ sơ đến khi nhận thư bảo lãnh đáp ứng kịp tiến độ hợp đồng.</t>
+          <t>Việc sửa đổi hoặc gia hạn thư bảo lãnh tại VietinBank được xử lý nhanh.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>SPEED4</t>
+          <t>DIGI1</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Việc sửa đổi hoặc gia hạn thư bảo lãnh tại VietinBank được xử lý nhanh.</t>
+          <t>Doanh nghiệp nộp được đề nghị cấp bảo lãnh trực tuyến qua VietinBank eFAST.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1184,12 +1184,12 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert)</t>
+          <t>1–5 (Likert); 9 = Chưa sử dụng (coi là khuyết)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>PROC_SPEED</t>
+          <t>DIGITAL_CONV</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1201,7 +1201,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>DIGI1</t>
+          <t>DIGI2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Doanh nghiệp nộp được đề nghị cấp bảo lãnh trực tuyến qua VietinBank eFAST.</t>
+          <t>VietinBank phát hành thư bảo lãnh điện tử có chữ ký số nhanh chóng.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1243,7 +1243,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>DIGI2</t>
+          <t>DIGI3</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>VietinBank phát hành thư bảo lãnh điện tử có chữ ký số nhanh chóng.</t>
+          <t>Việc tra cứu trạng thái hồ sơ bảo lãnh trực tuyến thuận tiện.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -1285,7 +1285,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DIGI3</t>
+          <t>DIGI4</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Việc tra cứu trạng thái hồ sơ bảo lãnh trực tuyến thuận tiện.</t>
+          <t>Bên thụ hưởng chấp nhận thư bảo lãnh điện tử của VietinBank mà không yêu cầu bản giấy.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>DIGI4</t>
+          <t>REPU1</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Bên thụ hưởng chấp nhận thư bảo lãnh điện tử của VietinBank mà không yêu cầu bản giấy.</t>
+          <t>VietinBank có uy tín thuộc nhóm dẫn đầu thị trường ngân hàng Việt Nam.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1352,12 +1352,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert); 9 = Chưa sử dụng (coi là khuyết)</t>
+          <t>1–5 (Likert)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>DIGITAL_CONV</t>
+          <t>BANK_REP</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -1369,7 +1369,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>REPU1</t>
+          <t>REPU2</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>VietinBank có uy tín thuộc nhóm dẫn đầu thị trường ngân hàng Việt Nam.</t>
+          <t>Thư bảo lãnh của VietinBank được chủ đầu tư và bên mời thầu chấp nhận rộng rãi.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>REPU2</t>
+          <t>REPU3</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Thư bảo lãnh của VietinBank được chủ đầu tư và bên mời thầu chấp nhận rộng rãi.</t>
+          <t>Năng lực tài chính của VietinBank tạo thêm uy tín cho Doanh nghiệp khi dự thầu.</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -1453,7 +1453,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>REPU3</t>
+          <t>REPU4</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Năng lực tài chính của VietinBank tạo thêm uy tín cho Doanh nghiệp khi dự thầu.</t>
+          <t>Doanh nghiệp yên tâm về khả năng VietinBank thực hiện nghĩa vụ khi thư bảo lãnh bị yêu cầu thanh toán.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1495,7 +1495,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>REPU4</t>
+          <t>RELA1</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Doanh nghiệp yên tâm về khả năng VietinBank thực hiện nghĩa vụ khi thư bảo lãnh bị yêu cầu thanh toán.</t>
+          <t>Quan hệ tín dụng lâu năm với VietinBank giúp Doanh nghiệp thuận lợi hơn khi đề nghị cấp bảo lãnh.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>BANK_REP</t>
+          <t>RELATIONSHIP</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -1537,7 +1537,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>RELA1</t>
+          <t>RELA2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Quan hệ tín dụng lâu năm với VietinBank giúp Doanh nghiệp thuận lợi hơn khi đề nghị cấp bảo lãnh.</t>
+          <t>Việc sử dụng các dịch vụ khác tại VietinBank mang lại ưu đãi cho hoạt động bảo lãnh.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>RELA2</t>
+          <t>RELA3</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Việc sử dụng các dịch vụ khác tại VietinBank mang lại ưu đãi cho hoạt động bảo lãnh.</t>
+          <t>VietinBank cấp hạn mức bảo lãnh phù hợp với nhu cầu của Doanh nghiệp.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>RELA3</t>
+          <t>RELA4</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>VietinBank cấp hạn mức bảo lãnh phù hợp với nhu cầu của Doanh nghiệp.</t>
+          <t>VietinBank điều chỉnh hạn mức kịp thời khi nhu cầu của Doanh nghiệp thay đổi.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1663,7 +1663,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>RELA4</t>
+          <t>STAFF1</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>VietinBank điều chỉnh hạn mức kịp thời khi nhu cầu của Doanh nghiệp thay đổi.</t>
+          <t>Cán bộ VietinBank có chuyên môn vững về nghiệp vụ bảo lãnh.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>RELATIONSHIP</t>
+          <t>STAFF_QUAL</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -1705,7 +1705,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>STAFF1</t>
+          <t>STAFF2</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank có chuyên môn vững về nghiệp vụ bảo lãnh.</t>
+          <t>Cán bộ VietinBank tư vấn được nội dung thư bảo lãnh phù hợp quy định pháp luật hiện hành.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>STAFF2</t>
+          <t>STAFF3</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank tư vấn được nội dung thư bảo lãnh phù hợp quy định pháp luật hiện hành.</t>
+          <t>Cán bộ VietinBank cảnh báo được các rủi ro trong điều khoản bảo lãnh trước khi phát hành.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -1789,7 +1789,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>STAFF3</t>
+          <t>STAFF4</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank cảnh báo được các rủi ro trong điều khoản bảo lãnh trước khi phát hành.</t>
+          <t>Cán bộ VietinBank phản hồi kịp thời khi Doanh nghiệp có vướng mắc.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1831,7 +1831,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>STAFF4</t>
+          <t>COLL1</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Cán bộ VietinBank phản hồi kịp thời khi Doanh nghiệp có vướng mắc.</t>
+          <t>VietinBank áp dụng tỷ lệ ký quỹ phù hợp với năng lực của Doanh nghiệp.</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>STAFF_QUAL</t>
+          <t>COLL_POLICY</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1873,7 +1873,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>COLL1</t>
+          <t>COLL2</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>VietinBank áp dụng tỷ lệ ký quỹ phù hợp với năng lực của Doanh nghiệp.</t>
+          <t>VietinBank có chính sách giảm hoặc miễn ký quỹ cho khách hàng đủ điều kiện.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>COLL2</t>
+          <t>COLL3</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>VietinBank có chính sách giảm hoặc miễn ký quỹ cho khách hàng đủ điều kiện.</t>
+          <t>VietinBank chấp nhận nhiều loại tài sản bảo đảm khác nhau.</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -1957,7 +1957,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>COLL3</t>
+          <t>COLL4</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>VietinBank chấp nhận nhiều loại tài sản bảo đảm khác nhau.</t>
+          <t>Thủ tục định giá và nhận tài sản bảo đảm tại VietinBank nhanh gọn.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1999,7 +1999,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>COLL4</t>
+          <t>DEC1</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Thủ tục định giá và nhận tài sản bảo đảm tại VietinBank nhanh gọn.</t>
+          <t>Khi phát sinh nhu cầu bảo lãnh, Doanh nghiệp ưu tiên lựa chọn VietinBank trước các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2029,19 +2029,19 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>COLL_POLICY</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>Biến quan sát — vào Cronbach's Alpha và EFA</t>
+          <t>Biến quan sát của biến phụ thuộc</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>DEC1</t>
+          <t>DEC2</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Khi phát sinh nhu cầu bảo lãnh, Doanh nghiệp ưu tiên lựa chọn VietinBank trước các ngân hàng khác.</t>
+          <t>Doanh nghiệp dành phần lớn giá trị bảo lãnh của mình cho VietinBank thay vì các ngân hàng khác.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2083,7 +2083,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>DEC2</t>
+          <t>DEC3</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -2093,7 +2093,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Doanh nghiệp dành phần lớn giá trị bảo lãnh của mình cho VietinBank thay vì các ngân hàng khác.</t>
+          <t>Trong các gói thầu và hợp đồng sắp tới, Doanh nghiệp dự định tiếp tục chọn VietinBank.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2125,7 +2125,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>DEC3</t>
+          <t>DEC4</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Trong các gói thầu và hợp đồng sắp tới, Doanh nghiệp dự định tiếp tục chọn VietinBank.</t>
+          <t>Doanh nghiệp sẵn sàng giới thiệu VietinBank cho đối tác như ngân hàng phát hành bảo lãnh tốt nhất.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2167,82 +2167,40 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>DEC4</t>
+          <t>WALLET_SHARE</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Phần C</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Doanh nghiệp sẵn sàng giới thiệu VietinBank cho đối tác như ngân hàng phát hành bảo lãnh tốt nhất.</t>
+          <t>Ước tính trong 12 tháng qua, VietinBank chiếm khoảng bao nhiêu phần trăm tổng giá trị bảo lãnh của Doanh nghiệp?</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Định lượng</t>
+          <t>Định tính</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Likert 5 mức</t>
+          <t>Thứ bậc</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>1–5 (Likert)</t>
+          <t>1 = Dưới 25%; 2 = Từ 25% đến 50%; 3 = Trên 50% đến 75%; 4 = Trên 75%</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Biến quan sát của biến phụ thuộc</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>WALLET_SHARE</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Ước tính trong 12 tháng qua, VietinBank chiếm khoảng bao nhiêu phần trăm tổng giá trị bảo lãnh của Doanh nghiệp?</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>Định tính</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Thứ bậc</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>1 = Dưới 25%; 2 = Từ 25% đến 50%; 3 = Trên 50% đến 75%; 4 = Trên 75%</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Biến đối chứng — tương quan Spearman với DEC để kiểm định giá trị tiêu chuẩn</t>
         </is>
@@ -2260,7 +2218,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -2600,7 +2558,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -2907,12 +2865,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Thêm biến giả D_SOE, D_FDI, D_LARGE, D_CONSTR</t>
+          <t>Thêm biến giả OWNERSHIP, REVENUE, NUM_BANKS</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Xác nhận β1–β7 ổn định; dùng D_CONSTR thay cho D_SINGLE tránh trùng DEC2</t>
+          <t>Xác nhận β1–β7 ổn định</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2892,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Nhóm có n &lt; 30 (Other) loại khỏi ANOVA</t>
+          <t>Nhóm có n &lt; 30 phải gộp trước khi chạy</t>
         </is>
       </c>
     </row>

</xml_diff>